<commit_message>
feat: support inventory-style card tables
</commit_message>
<xml_diff>
--- a/card-template.xlsx
+++ b/card-template.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="卡牌表" sheetId="1" r:id="Re71a5fd303744a5d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" r:id="R793c6071cf0e4431"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -13,44 +13,25 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <x:styleSheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <x:fonts count="3">
+  <x:numFmts count="1">
+    <x:numFmt numFmtId="200" formatCode="@"/>
+  </x:numFmts>
+  <x:fonts count="2">
     <x:font>
       <x:sz val="11"/>
       <x:name val="Carlito"/>
     </x:font>
     <x:font>
-      <x:b/>
-      <x:sz val="12"/>
-      <x:color rgb="FFFFFFFF"/>
-      <x:name val="Carlito"/>
-    </x:font>
-    <x:font>
       <x:sz val="11"/>
-      <x:color rgb="FF1F2937"/>
-      <x:name val="Carlito"/>
+      <x:name val="宋体"/>
     </x:font>
   </x:fonts>
-  <x:fills count="5">
+  <x:fills count="2">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
     <x:fill>
       <x:patternFill patternType="gray125"/>
-    </x:fill>
-    <x:fill>
-      <x:patternFill patternType="solid">
-        <x:fgColor rgb="FF1F2937"/>
-      </x:patternFill>
-    </x:fill>
-    <x:fill>
-      <x:patternFill patternType="solid">
-        <x:fgColor rgb="FFF8FAFC"/>
-      </x:patternFill>
-    </x:fill>
-    <x:fill>
-      <x:patternFill patternType="solid">
-        <x:fgColor rgb="FFE2E8F0"/>
-      </x:patternFill>
     </x:fill>
   </x:fills>
   <x:borders count="1">
@@ -59,26 +40,14 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="10">
+  <x:cellXfs count="4">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment horizontal="center"/>
+    <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
     </x:xf>
-    <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment horizontal="center" vertical="center"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <x:xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <x:xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment wrapText="1"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment vertical="top" wrapText="1"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="2" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment vertical="top" wrapText="1"/>
+    <x:xf numFmtId="200" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
     </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
@@ -282,39 +251,91 @@
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
-    <x:col min="1" max="1" width="22" hidden="0" customWidth="1"/>
-    <x:col min="2" max="2" width="58" hidden="0" customWidth="1"/>
+    <x:col min="1" max="1" width="9.375" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="37.375" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="15" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="7" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="8.875" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="87.25" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
-    <x:row r="1" ht="28" customHeight="1">
-      <x:c r="A1" s="4" t="str">
-        <x:v>名称</x:v>
-      </x:c>
-      <x:c r="B1" s="4" t="str">
-        <x:v>内容</x:v>
+    <x:row r="1">
+      <x:c r="A1" s="3" t="str">
+        <x:v>快递编号</x:v>
+      </x:c>
+      <x:c r="B1" s="2" t="str">
+        <x:v>物品名称</x:v>
+      </x:c>
+      <x:c r="C1" s="2" t="str">
+        <x:v>发件地</x:v>
+      </x:c>
+      <x:c r="D1" s="2" t="str">
+        <x:v>收件人</x:v>
+      </x:c>
+      <x:c r="E1" s="2" t="str">
+        <x:v>物品类型</x:v>
+      </x:c>
+      <x:c r="F1" s="2" t="str">
+        <x:v>附加文本</x:v>
       </x:c>
     </x:row>
-    <x:row r="2" ht="36" customHeight="1">
-      <x:c r="A2" s="8" t="str">
+    <x:row r="2">
+      <x:c r="A2" s="3" t="str">
+        <x:v>A-M-0001</x:v>
+      </x:c>
+      <x:c r="B2" s="2" t="str">
         <x:v>医疗箱</x:v>
       </x:c>
-      <x:c r="B2" s="8" t="str">
+      <x:c r="C2" s="2" t="str">
+        <x:v>山东青岛</x:v>
+      </x:c>
+      <x:c r="D2" s="2" t="str">
+        <x:v>许泽洋</x:v>
+      </x:c>
+      <x:c r="E2" s="2" t="str">
+        <x:v>医疗</x:v>
+      </x:c>
+      <x:c r="F2" s="2" t="str">
         <x:v>获得基础治疗物资。</x:v>
       </x:c>
     </x:row>
-    <x:row r="3" ht="36" customHeight="1">
-      <x:c r="A3" s="9" t="str">
+    <x:row r="3">
+      <x:c r="A3" s="3" t="str">
+        <x:v>A-L-0002</x:v>
+      </x:c>
+      <x:c r="B3" s="2" t="str">
         <x:v>沾血的收据</x:v>
       </x:c>
-      <x:c r="B3" s="9" t="str">
+      <x:c r="C3" s="2" t="str">
+        <x:v>河北廊坊</x:v>
+      </x:c>
+      <x:c r="D3" s="2" t="str">
+        <x:v>王浩</x:v>
+      </x:c>
+      <x:c r="E3" s="2" t="str">
+        <x:v>线索</x:v>
+      </x:c>
+      <x:c r="F3" s="2" t="str">
         <x:v>记录着一个尚未搜查的地址。</x:v>
       </x:c>
     </x:row>
-    <x:row r="4" ht="36" customHeight="1">
-      <x:c r="A4" s="8" t="str">
+    <x:row r="4">
+      <x:c r="A4" s="3" t="str">
+        <x:v>A-L-0003</x:v>
+      </x:c>
+      <x:c r="B4" s="2" t="str">
         <x:v>封死的保温箱</x:v>
       </x:c>
-      <x:c r="B4" s="8" t="str">
+      <x:c r="C4" s="2" t="str">
+        <x:v>辽宁沈阳</x:v>
+      </x:c>
+      <x:c r="D4" s="2" t="str">
+        <x:v>刘雨桐</x:v>
+      </x:c>
+      <x:c r="E4" s="2" t="str">
+        <x:v>事件</x:v>
+      </x:c>
+      <x:c r="F4" s="2" t="str">
         <x:v>里面传来微弱的抓挠声。</x:v>
       </x:c>
     </x:row>

</xml_diff>